<commit_message>
Rewrite 365 calendar hooks and regenerate review documents
</commit_message>
<xml_diff>
--- a/review/etnografiya/april/april.xlsx
+++ b/review/etnografiya/april/april.xlsx
@@ -108,7 +108,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Этой деревянной лопаткой не готовили еду. Что она делала у воды?</t>
+          <t xml:space="preserve">Деревянной лопаткой работают у воды, а не у плиты. Валёк помогает стирать бельё: знакомая форма скрывает другую домашнюю нагрузку.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -135,7 +135,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Почему у обыкновенной стиральной доски есть автор?</t>
+          <t xml:space="preserve">У стиральной доски есть конкретный изготовитель. Даже привычная домашняя вещь сохраняет авторство и след труда, который обычно остаётся незаметным.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -162,7 +162,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Как получить большую ёмкость, если нет ни досок, ни обручей?</t>
+          <t xml:space="preserve">Большую ёмкость выдалбливают из цельного дерева. Ни досок, ни обручей — стенки и дно остаются частями одной заготовки.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -189,7 +189,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Как одним маленьким колёсиком сделать комнату светлее?</t>
+          <t xml:space="preserve">Маленькое колёсико меняет положение фитиля. Свет керосиновой лампы зависит от движения детали, которую легко не заметить рядом со стеклом.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -216,7 +216,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Почему праздник о далёком Иерусалиме встречают с вербой?</t>
+          <t xml:space="preserve">Праздник Входа в Иерусалим встречают с вербой. Весенняя ветвь входит в русскую местную традицию праздника с далёким евангельским событием.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -243,7 +243,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Зачем украшать ту сторону деревянной формы, которую никто не видит?</t>
+          <t xml:space="preserve">Узор внутри пасочницы появится снаружи на готовой пасхе. Скрытая резьба формы работает как обратное изображение будущего праздничного блюда.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -270,7 +270,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Что важнее привычной работы, если даже прялку оставляют в покое?</t>
+          <t xml:space="preserve">На Благовещение привычную работу могли откладывать. Остановленная прялка становится знаком праздничного времени в народном домашнем укладе.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -297,7 +297,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Может ли маленький подарок рассказать, кто и кому его поднёс?</t>
+          <t xml:space="preserve">Маленький пасхальный подарок хранит адресное обращение. Надпись и отделка помогают увидеть за вещью человека, который выбирал её для другого.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -324,7 +324,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Как выиграть пасхальное яйцо, не разбивая его?</t>
+          <t xml:space="preserve">Пасхальное яйцо можно выиграть катанием. Праздничная игра требует рассчитать путь целой хрупкой вещи, не превращая встречу в бой скорлупок.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -351,7 +351,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Как поздравить человека, до которого нельзя дойти пешком?</t>
+          <t xml:space="preserve">Праздничная открытка проходит дорогу вместо отправителя. Подпись соединяет людей, которые не могут встретиться за одним столом.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -378,7 +378,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Зачем к чаепитию понадобились кусачки с маленьким поддоном?</t>
+          <t xml:space="preserve">Кусачки отделяют кусочек от сахарной головы. Маленький поддон у инструмента напоминает, что сладкое угощение когда-то готовили иначе.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -405,7 +405,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Как рассказать о духовном пути при помощи теста?</t>
+          <t xml:space="preserve">Лестница из теста становится образом духовного пути. Домашняя выпечка сохраняет символ праздника в предмете, который можно взять в руки.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -432,7 +432,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Куда делся кофе, если зёрна засыпали сверху?</t>
+          <t xml:space="preserve">Зёрна засыпают сверху, молотый кофе собирается внизу. Между ними работает ручной механизм — чашка начинается с усилия человека.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -459,7 +459,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Почему тяжёлую чугунную вещь помнят по тарелке вафель?</t>
+          <t xml:space="preserve">Тяжёлую чугунную вафельницу помнят по лёгкому хрустящему угощению. Рельеф горячих створок остаётся рисунком на готовой выпечке.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -486,7 +486,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Как везти чернила с собой, когда ручку ещё надо обмакивать?</t>
+          <t xml:space="preserve">Чернила берут в дорогу в отдельной вещи. Походная чернильница хранит время, когда пишущий инструмент приходилось снова обмакивать.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -513,7 +513,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Что в названии народного дня напоминает о движении воды?</t>
+          <t xml:space="preserve">Народное имя весеннего дня напоминает о движении воды. За названием стоит наблюдение за сезонной переменой, а не точная дата ледохода.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -540,7 +540,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Что делали с телефоном, у которого нет привычного набора номера?</t>
+          <t xml:space="preserve">У старого телефона нет привычного набора номера. Связь начиналась с другого действия — устройство показывает перемены в повседневном общении.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Как освободить руки, когда несёшь всё нужное через лес?</t>
+          <t xml:space="preserve">Кузовок освобождает руки в лесной дороге. Плетёная вещь распределяет ношу за спиной и соединяет свойства материала с движением человека.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -594,7 +594,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Почему много деревянных пальцев делают работу быстрее одного?</t>
+          <t xml:space="preserve">Много деревянных зубьев работают одним движением. Грабли собирают рассеянное по земле — ширина инструмента превращает усилие в быстрый проход.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Как передать усилие лошади повозке и распределить контакт с телом?</t>
+          <t xml:space="preserve">Хомут соединяет тело лошади с работой повозки. Форма упряжи распределяет контакт и передаёт тягу: удобство здесь связано с устройством.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -648,7 +648,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Почему работа с деревом стала выражением о безделье?</t>
+          <t xml:space="preserve">Баклуша — деревянная заготовка, а выражение звучит как безделье. За знакомыми словами скрыт реальный этап изготовления домашней утвари.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Почему сапожнику нужна ещё одна нога, кроме ноги заказчика?</t>
+          <t xml:space="preserve">Сапожник работает с колодкой вместо ноги заказчика. Деревянная форма удерживает размер и объём, пока плоский материал становится обувью.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Может ли рабочий сигнал превратиться в мелодию для гулянья?</t>
+          <t xml:space="preserve">Пастушеский рожок подаёт сигнал и звучит в музыкальном ансамбле. Рабочий инструмент получает новую жизнь в руках исполнителя.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Почему привычному гармонисту бывает трудно сыграть на другой гармони?</t>
+          <t xml:space="preserve">Привычные движения не всегда подходят другой гармони. Местные системы инструмента сохраняют разные способы извлекать и связывать звуки.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Что должен сделать мастер, чтобы знакомый инструмент зазвучал в оркестре?</t>
+          <t xml:space="preserve">Для оркестра знакомый инструмент меняют и настраивают. Работа мастера помогает народному звучанию войти в согласованный голос большого состава.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Что меняется в празднике, когда человек сам входит в хоровод?</t>
+          <t xml:space="preserve">Человек входит в хоровод и становится частью общего движения. Праздник складывается из согласованного шага, пения и внимания к соседу.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Почему народный хор не звучит как несколько одинаковых голосов?</t>
+          <t xml:space="preserve">Народный хор объединяет разные голоса. Общее звучание возникает из их взаимодействия — отдельная партия не обязана повторять остальные.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Почему детская игровая бита отлита из чугуна и украшена?</t>
+          <t xml:space="preserve">Игровая бита отлита из чугуна и украшена. Маленькая детская вещь хранит вес настоящего материала и внимание мастера к её виду.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Как устроить музыкальный вечер там, где нет розетки?</t>
+          <t xml:space="preserve">Музыкальный вечер начинается без розетки. Заведённый механизм граммофона двигает пластинку — домашнее слушание имеет собственную историю труда.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Можно ли вытащить крошечную расписную вещь, не потревожив остальные?</t>
+          <t xml:space="preserve">Из расписной вещи появляется ещё одна, меньше. Матрёшка держит целую последовательность объёмов внутри формы, которая кажется одной игрушкой.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">

</xml_diff>